<commit_message>
Update manuscript submission package and consolidate analysis outputs
</commit_message>
<xml_diff>
--- a/data/phenology_data/phenology.xlsx
+++ b/data/phenology_data/phenology.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yaolinjia/Desktop/Grape/dm_first_inf/data/phenology_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{603A15AE-6121-AB40-9CED-D843D3DA1963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B107F3B-3830-A242-B82B-11448884E5C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{1D63C8CD-29E1-2F4D-8B98-B68AE6EDFD36}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16860" xr2:uid="{1D63C8CD-29E1-2F4D-8B98-B68AE6EDFD36}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="9">
   <si>
     <t>latitude</t>
   </si>
@@ -127,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -149,6 +149,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -484,13 +487,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EF35035-13FE-0B46-AA69-038A959D6429}">
-  <dimension ref="A1:F77"/>
+  <dimension ref="A1:J80"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="16384" width="10.83203125" style="2"/>
+    <col min="1" max="6" width="10.83203125" style="2"/>
+    <col min="8" max="16384" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>5</v>
       </c>
@@ -510,7 +514,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>6</v>
       </c>
@@ -524,53 +528,54 @@
         <v>2023</v>
       </c>
       <c r="E2" s="3">
+        <v>44991</v>
+      </c>
+      <c r="F2" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="1">
+        <v>22.61</v>
+      </c>
+      <c r="C3" s="1">
+        <v>108.23</v>
+      </c>
+      <c r="D3" s="1">
+        <v>2023</v>
+      </c>
+      <c r="E3" s="3">
         <v>44999</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F3" s="1">
         <v>13</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="1">
-        <v>22.61</v>
-      </c>
-      <c r="C3" s="1">
-        <v>108.23</v>
-      </c>
-      <c r="D3" s="1">
-        <v>2023</v>
-      </c>
-      <c r="E3" s="3">
+      <c r="J3" s="8"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1">
+        <v>22.61</v>
+      </c>
+      <c r="C4" s="1">
+        <v>108.23</v>
+      </c>
+      <c r="D4" s="1">
+        <v>2023</v>
+      </c>
+      <c r="E4" s="3">
         <v>45006</v>
-      </c>
-      <c r="F3" s="1">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="1">
-        <v>22.61</v>
-      </c>
-      <c r="C4" s="1">
-        <v>108.23</v>
-      </c>
-      <c r="D4" s="1">
-        <v>2023</v>
-      </c>
-      <c r="E4" s="3">
-        <v>45009</v>
       </c>
       <c r="F4" s="1">
         <v>55</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>6</v>
       </c>
@@ -584,33 +589,33 @@
         <v>2023</v>
       </c>
       <c r="E5" s="3">
+        <v>45009</v>
+      </c>
+      <c r="F5" s="1">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="1">
+        <v>22.61</v>
+      </c>
+      <c r="C6" s="1">
+        <v>108.23</v>
+      </c>
+      <c r="D6" s="1">
+        <v>2023</v>
+      </c>
+      <c r="E6" s="3">
         <v>45012</v>
-      </c>
-      <c r="F5" s="1">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="1">
-        <v>22.61</v>
-      </c>
-      <c r="C6" s="1">
-        <v>108.23</v>
-      </c>
-      <c r="D6" s="1">
-        <v>2023</v>
-      </c>
-      <c r="E6" s="3">
-        <v>45015</v>
       </c>
       <c r="F6" s="1">
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>6</v>
       </c>
@@ -624,13 +629,13 @@
         <v>2023</v>
       </c>
       <c r="E7" s="3">
-        <v>45018</v>
+        <v>45015</v>
       </c>
       <c r="F7" s="1">
         <v>57</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>6</v>
       </c>
@@ -644,13 +649,13 @@
         <v>2023</v>
       </c>
       <c r="E8" s="3">
-        <v>45021</v>
+        <v>45018</v>
       </c>
       <c r="F8" s="1">
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>6</v>
       </c>
@@ -664,13 +669,13 @@
         <v>2023</v>
       </c>
       <c r="E9" s="3">
-        <v>45024</v>
+        <v>45021</v>
       </c>
       <c r="F9" s="1">
         <v>57</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
         <v>6</v>
       </c>
@@ -684,73 +689,73 @@
         <v>2023</v>
       </c>
       <c r="E10" s="3">
+        <v>45024</v>
+      </c>
+      <c r="F10" s="1">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A11" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" s="1">
+        <v>22.61</v>
+      </c>
+      <c r="C11" s="1">
+        <v>108.23</v>
+      </c>
+      <c r="D11" s="1">
+        <v>2023</v>
+      </c>
+      <c r="E11" s="3">
         <v>45027</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F11" s="1">
         <v>65</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B11" s="1">
-        <v>22.61</v>
-      </c>
-      <c r="C11" s="1">
-        <v>108.23</v>
-      </c>
-      <c r="D11" s="1">
-        <v>2023</v>
-      </c>
-      <c r="E11" s="3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A12" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B12" s="1">
+        <v>22.61</v>
+      </c>
+      <c r="C12" s="1">
+        <v>108.23</v>
+      </c>
+      <c r="D12" s="1">
+        <v>2023</v>
+      </c>
+      <c r="E12" s="3">
         <v>45030</v>
       </c>
-      <c r="F11" s="1">
+      <c r="F12" s="1">
         <v>68</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B12" s="1">
-        <v>22.61</v>
-      </c>
-      <c r="C12" s="1">
-        <v>108.23</v>
-      </c>
-      <c r="D12" s="1">
-        <v>2023</v>
-      </c>
-      <c r="E12" s="3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A13" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B13" s="1">
+        <v>22.61</v>
+      </c>
+      <c r="C13" s="1">
+        <v>108.23</v>
+      </c>
+      <c r="D13" s="1">
+        <v>2023</v>
+      </c>
+      <c r="E13" s="3">
         <v>45033</v>
-      </c>
-      <c r="F12" s="1">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B13" s="1">
-        <v>22.61</v>
-      </c>
-      <c r="C13" s="1">
-        <v>108.23</v>
-      </c>
-      <c r="D13" s="1">
-        <v>2023</v>
-      </c>
-      <c r="E13" s="3">
-        <v>45036</v>
       </c>
       <c r="F13" s="1">
         <v>73</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
         <v>6</v>
       </c>
@@ -764,13 +769,13 @@
         <v>2023</v>
       </c>
       <c r="E14" s="3">
-        <v>45039</v>
+        <v>45036</v>
       </c>
       <c r="F14" s="1">
         <v>73</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
         <v>6</v>
       </c>
@@ -784,13 +789,13 @@
         <v>2023</v>
       </c>
       <c r="E15" s="3">
-        <v>45042</v>
+        <v>45039</v>
       </c>
       <c r="F15" s="1">
         <v>73</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
         <v>6</v>
       </c>
@@ -804,53 +809,53 @@
         <v>2023</v>
       </c>
       <c r="E16" s="3">
+        <v>45042</v>
+      </c>
+      <c r="F16" s="1">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A17" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B17" s="1">
+        <v>22.61</v>
+      </c>
+      <c r="C17" s="1">
+        <v>108.23</v>
+      </c>
+      <c r="D17" s="1">
+        <v>2023</v>
+      </c>
+      <c r="E17" s="3">
         <v>45045</v>
       </c>
-      <c r="F16" s="1">
+      <c r="F17" s="1">
         <v>77</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B17" s="1">
-        <v>22.61</v>
-      </c>
-      <c r="C17" s="1">
-        <v>108.23</v>
-      </c>
-      <c r="D17" s="1">
-        <v>2023</v>
-      </c>
-      <c r="E17" s="3">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A18" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B18" s="1">
+        <v>22.61</v>
+      </c>
+      <c r="C18" s="1">
+        <v>108.23</v>
+      </c>
+      <c r="D18" s="1">
+        <v>2023</v>
+      </c>
+      <c r="E18" s="3">
         <v>45048</v>
-      </c>
-      <c r="F17" s="1">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A18" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B18" s="1">
-        <v>22.61</v>
-      </c>
-      <c r="C18" s="1">
-        <v>108.23</v>
-      </c>
-      <c r="D18" s="1">
-        <v>2023</v>
-      </c>
-      <c r="E18" s="3">
-        <v>45051</v>
       </c>
       <c r="F18" s="1">
         <v>79</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
         <v>6</v>
       </c>
@@ -864,13 +869,13 @@
         <v>2023</v>
       </c>
       <c r="E19" s="3">
-        <v>45054</v>
+        <v>45051</v>
       </c>
       <c r="F19" s="1">
         <v>79</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
         <v>6</v>
       </c>
@@ -884,13 +889,13 @@
         <v>2023</v>
       </c>
       <c r="E20" s="3">
-        <v>45057</v>
+        <v>45054</v>
       </c>
       <c r="F20" s="1">
         <v>79</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
         <v>6</v>
       </c>
@@ -904,193 +909,194 @@
         <v>2023</v>
       </c>
       <c r="E21" s="3">
+        <v>45057</v>
+      </c>
+      <c r="F21" s="1">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A22" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B22" s="1">
+        <v>22.61</v>
+      </c>
+      <c r="C22" s="1">
+        <v>108.23</v>
+      </c>
+      <c r="D22" s="1">
+        <v>2023</v>
+      </c>
+      <c r="E22" s="3">
         <v>45075</v>
       </c>
-      <c r="F21" s="1">
+      <c r="F22" s="1">
         <v>81</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A22" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B22" s="1">
-        <v>22.61</v>
-      </c>
-      <c r="C22" s="1">
-        <v>108.23</v>
-      </c>
-      <c r="D22" s="1">
-        <v>2024</v>
-      </c>
-      <c r="E22" s="3">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A23" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B23" s="1">
+        <v>22.61</v>
+      </c>
+      <c r="C23" s="1">
+        <v>108.23</v>
+      </c>
+      <c r="D23" s="1">
+        <v>2024</v>
+      </c>
+      <c r="E23" s="3">
+        <v>45369</v>
+      </c>
+      <c r="F23" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A24" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B24" s="1">
+        <v>22.61</v>
+      </c>
+      <c r="C24" s="1">
+        <v>108.23</v>
+      </c>
+      <c r="D24" s="1">
+        <v>2024</v>
+      </c>
+      <c r="E24" s="3">
         <v>45383</v>
       </c>
-      <c r="F22" s="1">
+      <c r="F24" s="1">
         <v>15</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A23" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B23" s="1">
-        <v>22.61</v>
-      </c>
-      <c r="C23" s="1">
-        <v>108.23</v>
-      </c>
-      <c r="D23" s="1">
-        <v>2024</v>
-      </c>
-      <c r="E23" s="3">
+      <c r="J24" s="8"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A25" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B25" s="1">
+        <v>22.61</v>
+      </c>
+      <c r="C25" s="1">
+        <v>108.23</v>
+      </c>
+      <c r="D25" s="1">
+        <v>2024</v>
+      </c>
+      <c r="E25" s="3">
         <v>45386</v>
       </c>
-      <c r="F23" s="1">
+      <c r="F25" s="1">
         <v>53</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A24" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B24" s="1">
-        <v>22.61</v>
-      </c>
-      <c r="C24" s="1">
-        <v>108.23</v>
-      </c>
-      <c r="D24" s="1">
-        <v>2024</v>
-      </c>
-      <c r="E24" s="3">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A26" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B26" s="1">
+        <v>22.61</v>
+      </c>
+      <c r="C26" s="1">
+        <v>108.23</v>
+      </c>
+      <c r="D26" s="1">
+        <v>2024</v>
+      </c>
+      <c r="E26" s="3">
         <v>45389</v>
       </c>
-      <c r="F24" s="1">
+      <c r="F26" s="1">
         <v>55</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A25" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B25" s="1">
-        <v>22.61</v>
-      </c>
-      <c r="C25" s="1">
-        <v>108.23</v>
-      </c>
-      <c r="D25" s="1">
-        <v>2024</v>
-      </c>
-      <c r="E25" s="3">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A27" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B27" s="1">
+        <v>22.61</v>
+      </c>
+      <c r="C27" s="1">
+        <v>108.23</v>
+      </c>
+      <c r="D27" s="1">
+        <v>2024</v>
+      </c>
+      <c r="E27" s="3">
         <v>45392</v>
       </c>
-      <c r="F25" s="1">
+      <c r="F27" s="1">
         <v>57</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A26" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B26" s="1">
-        <v>22.61</v>
-      </c>
-      <c r="C26" s="1">
-        <v>108.23</v>
-      </c>
-      <c r="D26" s="1">
-        <v>2024</v>
-      </c>
-      <c r="E26" s="3">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A28" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B28" s="1">
+        <v>22.61</v>
+      </c>
+      <c r="C28" s="1">
+        <v>108.23</v>
+      </c>
+      <c r="D28" s="1">
+        <v>2024</v>
+      </c>
+      <c r="E28" s="3">
         <v>45395</v>
       </c>
-      <c r="F26" s="1">
+      <c r="F28" s="1">
         <v>57</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A27" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B27" s="1">
-        <v>22.61</v>
-      </c>
-      <c r="C27" s="1">
-        <v>108.23</v>
-      </c>
-      <c r="D27" s="1">
-        <v>2024</v>
-      </c>
-      <c r="E27" s="3">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A29" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B29" s="1">
+        <v>22.61</v>
+      </c>
+      <c r="C29" s="1">
+        <v>108.23</v>
+      </c>
+      <c r="D29" s="1">
+        <v>2024</v>
+      </c>
+      <c r="E29" s="3">
         <v>45398</v>
       </c>
-      <c r="F27" s="1">
+      <c r="F29" s="1">
         <v>65</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A28" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B28" s="1">
-        <v>22.61</v>
-      </c>
-      <c r="C28" s="1">
-        <v>108.23</v>
-      </c>
-      <c r="D28" s="1">
-        <v>2024</v>
-      </c>
-      <c r="E28" s="3">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A30" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B30" s="1">
+        <v>22.61</v>
+      </c>
+      <c r="C30" s="1">
+        <v>108.23</v>
+      </c>
+      <c r="D30" s="1">
+        <v>2024</v>
+      </c>
+      <c r="E30" s="3">
         <v>45401</v>
-      </c>
-      <c r="F28" s="1">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A29" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B29" s="1">
-        <v>22.61</v>
-      </c>
-      <c r="C29" s="1">
-        <v>108.23</v>
-      </c>
-      <c r="D29" s="1">
-        <v>2024</v>
-      </c>
-      <c r="E29" s="3">
-        <v>45404</v>
-      </c>
-      <c r="F29" s="1">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A30" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B30" s="1">
-        <v>22.61</v>
-      </c>
-      <c r="C30" s="1">
-        <v>108.23</v>
-      </c>
-      <c r="D30" s="1">
-        <v>2024</v>
-      </c>
-      <c r="E30" s="3">
-        <v>45407</v>
       </c>
       <c r="F30" s="1">
         <v>71</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
         <v>6</v>
       </c>
@@ -1104,13 +1110,13 @@
         <v>2024</v>
       </c>
       <c r="E31" s="3">
-        <v>45410</v>
+        <v>45404</v>
       </c>
       <c r="F31" s="1">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
         <v>6</v>
       </c>
@@ -1124,10 +1130,10 @@
         <v>2024</v>
       </c>
       <c r="E32" s="3">
-        <v>45419</v>
+        <v>45407</v>
       </c>
       <c r="F32" s="1">
-        <v>79</v>
+        <v>71</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
@@ -1144,50 +1150,50 @@
         <v>2024</v>
       </c>
       <c r="E33" s="3">
-        <v>45445</v>
+        <v>45410</v>
       </c>
       <c r="F33" s="1">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B34" s="1">
-        <v>23.83</v>
+        <v>22.61</v>
       </c>
       <c r="C34" s="1">
-        <v>108.1</v>
+        <v>108.23</v>
       </c>
       <c r="D34" s="1">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="E34" s="3">
-        <v>44656</v>
+        <v>45419</v>
       </c>
       <c r="F34" s="1">
-        <v>9</v>
+        <v>79</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B35" s="1">
-        <v>23.83</v>
+        <v>22.61</v>
       </c>
       <c r="C35" s="1">
-        <v>108.1</v>
+        <v>108.23</v>
       </c>
       <c r="D35" s="1">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="E35" s="3">
-        <v>44698</v>
+        <v>45445</v>
       </c>
       <c r="F35" s="1">
-        <v>57</v>
+        <v>81</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
@@ -1204,10 +1210,10 @@
         <v>2022</v>
       </c>
       <c r="E36" s="3">
-        <v>44707</v>
+        <v>44656</v>
       </c>
       <c r="F36" s="1">
-        <v>65</v>
+        <v>9</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
@@ -1221,13 +1227,13 @@
         <v>108.1</v>
       </c>
       <c r="D37" s="1">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="E37" s="3">
-        <v>44999</v>
+        <v>44698</v>
       </c>
       <c r="F37" s="1">
-        <v>0</v>
+        <v>57</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
@@ -1241,13 +1247,13 @@
         <v>108.1</v>
       </c>
       <c r="D38" s="1">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="E38" s="3">
-        <v>45006</v>
+        <v>44707</v>
       </c>
       <c r="F38" s="1">
-        <v>0</v>
+        <v>65</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
@@ -1264,10 +1270,10 @@
         <v>2023</v>
       </c>
       <c r="E39" s="3">
-        <v>45013</v>
+        <v>44999</v>
       </c>
       <c r="F39" s="1">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
@@ -1284,10 +1290,10 @@
         <v>2023</v>
       </c>
       <c r="E40" s="3">
-        <v>45017</v>
+        <v>45006</v>
       </c>
       <c r="F40" s="1">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
@@ -1304,10 +1310,10 @@
         <v>2023</v>
       </c>
       <c r="E41" s="3">
-        <v>45020</v>
+        <v>45013</v>
       </c>
       <c r="F41" s="1">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
@@ -1324,10 +1330,10 @@
         <v>2023</v>
       </c>
       <c r="E42" s="3">
-        <v>45023</v>
+        <v>45017</v>
       </c>
       <c r="F42" s="1">
-        <v>53</v>
+        <v>9</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
@@ -1344,10 +1350,10 @@
         <v>2023</v>
       </c>
       <c r="E43" s="3">
-        <v>45026</v>
+        <v>45020</v>
       </c>
       <c r="F43" s="1">
-        <v>53</v>
+        <v>12</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
@@ -1364,10 +1370,10 @@
         <v>2023</v>
       </c>
       <c r="E44" s="3">
-        <v>45029</v>
+        <v>45023</v>
       </c>
       <c r="F44" s="1">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
@@ -1384,10 +1390,10 @@
         <v>2023</v>
       </c>
       <c r="E45" s="3">
-        <v>45032</v>
+        <v>45026</v>
       </c>
       <c r="F45" s="1">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
@@ -1404,7 +1410,7 @@
         <v>2023</v>
       </c>
       <c r="E46" s="3">
-        <v>45035</v>
+        <v>45029</v>
       </c>
       <c r="F46" s="1">
         <v>55</v>
@@ -1424,7 +1430,7 @@
         <v>2023</v>
       </c>
       <c r="E47" s="3">
-        <v>45038</v>
+        <v>45032</v>
       </c>
       <c r="F47" s="1">
         <v>55</v>
@@ -1444,10 +1450,10 @@
         <v>2023</v>
       </c>
       <c r="E48" s="3">
-        <v>45041</v>
+        <v>45035</v>
       </c>
       <c r="F48" s="1">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.2">
@@ -1464,10 +1470,10 @@
         <v>2023</v>
       </c>
       <c r="E49" s="3">
-        <v>45044</v>
+        <v>45038</v>
       </c>
       <c r="F49" s="1">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.2">
@@ -1484,7 +1490,7 @@
         <v>2023</v>
       </c>
       <c r="E50" s="3">
-        <v>45047</v>
+        <v>45041</v>
       </c>
       <c r="F50" s="1">
         <v>57</v>
@@ -1504,7 +1510,7 @@
         <v>2023</v>
       </c>
       <c r="E51" s="3">
-        <v>45050</v>
+        <v>45044</v>
       </c>
       <c r="F51" s="1">
         <v>57</v>
@@ -1524,7 +1530,7 @@
         <v>2023</v>
       </c>
       <c r="E52" s="3">
-        <v>45053</v>
+        <v>45047</v>
       </c>
       <c r="F52" s="1">
         <v>57</v>
@@ -1544,7 +1550,7 @@
         <v>2023</v>
       </c>
       <c r="E53" s="3">
-        <v>45056</v>
+        <v>45050</v>
       </c>
       <c r="F53" s="1">
         <v>57</v>
@@ -1564,10 +1570,10 @@
         <v>2023</v>
       </c>
       <c r="E54" s="3">
-        <v>45059</v>
+        <v>45053</v>
       </c>
       <c r="F54" s="1">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.2">
@@ -1584,10 +1590,10 @@
         <v>2023</v>
       </c>
       <c r="E55" s="3">
-        <v>45066</v>
+        <v>45056</v>
       </c>
       <c r="F55" s="1">
-        <v>65</v>
+        <v>57</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.2">
@@ -1604,10 +1610,10 @@
         <v>2023</v>
       </c>
       <c r="E56" s="3">
-        <v>45078</v>
+        <v>45059</v>
       </c>
       <c r="F56" s="1">
-        <v>71</v>
+        <v>61</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.2">
@@ -1621,13 +1627,13 @@
         <v>108.1</v>
       </c>
       <c r="D57" s="1">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="E57" s="3">
-        <v>45384</v>
+        <v>45066</v>
       </c>
       <c r="F57" s="1">
-        <v>9</v>
+        <v>65</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.2">
@@ -1641,13 +1647,13 @@
         <v>108.1</v>
       </c>
       <c r="D58" s="1">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="E58" s="3">
-        <v>45391</v>
+        <v>45078</v>
       </c>
       <c r="F58" s="1">
-        <v>53</v>
+        <v>71</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.2">
@@ -1664,10 +1670,10 @@
         <v>2024</v>
       </c>
       <c r="E59" s="3">
-        <v>45394</v>
+        <v>45384</v>
       </c>
       <c r="F59" s="1">
-        <v>53</v>
+        <v>9</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.2">
@@ -1684,10 +1690,10 @@
         <v>2024</v>
       </c>
       <c r="E60" s="3">
-        <v>45397</v>
+        <v>45391</v>
       </c>
       <c r="F60" s="1">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.2">
@@ -1704,10 +1710,10 @@
         <v>2024</v>
       </c>
       <c r="E61" s="3">
-        <v>45400</v>
+        <v>45394</v>
       </c>
       <c r="F61" s="1">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.2">
@@ -1724,10 +1730,10 @@
         <v>2024</v>
       </c>
       <c r="E62" s="3">
-        <v>45403</v>
+        <v>45397</v>
       </c>
       <c r="F62" s="1">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.2">
@@ -1744,10 +1750,10 @@
         <v>2024</v>
       </c>
       <c r="E63" s="3">
-        <v>45406</v>
+        <v>45400</v>
       </c>
       <c r="F63" s="1">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.2">
@@ -1764,13 +1770,13 @@
         <v>2024</v>
       </c>
       <c r="E64" s="3">
-        <v>45409</v>
+        <v>45403</v>
       </c>
       <c r="F64" s="1">
         <v>57</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A65" s="5" t="s">
         <v>7</v>
       </c>
@@ -1784,13 +1790,13 @@
         <v>2024</v>
       </c>
       <c r="E65" s="3">
-        <v>45415</v>
+        <v>45406</v>
       </c>
       <c r="F65" s="1">
         <v>57</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A66" s="5" t="s">
         <v>7</v>
       </c>
@@ -1804,113 +1810,113 @@
         <v>2024</v>
       </c>
       <c r="E66" s="3">
+        <v>45409</v>
+      </c>
+      <c r="F66" s="1">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A67" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B67" s="1">
+        <v>23.83</v>
+      </c>
+      <c r="C67" s="1">
+        <v>108.1</v>
+      </c>
+      <c r="D67" s="1">
+        <v>2024</v>
+      </c>
+      <c r="E67" s="3">
+        <v>45415</v>
+      </c>
+      <c r="F67" s="1">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A68" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B68" s="1">
+        <v>23.83</v>
+      </c>
+      <c r="C68" s="1">
+        <v>108.1</v>
+      </c>
+      <c r="D68" s="1">
+        <v>2024</v>
+      </c>
+      <c r="E68" s="3">
         <v>45418</v>
       </c>
-      <c r="F66" s="1">
+      <c r="F68" s="1">
         <v>61</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A67" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B67" s="1">
-        <v>23.83</v>
-      </c>
-      <c r="C67" s="1">
-        <v>108.1</v>
-      </c>
-      <c r="D67" s="1">
-        <v>2024</v>
-      </c>
-      <c r="E67" s="3">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A69" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B69" s="1">
+        <v>23.83</v>
+      </c>
+      <c r="C69" s="1">
+        <v>108.1</v>
+      </c>
+      <c r="D69" s="1">
+        <v>2024</v>
+      </c>
+      <c r="E69" s="3">
         <v>45430</v>
       </c>
-      <c r="F67" s="1">
+      <c r="F69" s="1">
         <v>65</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A68" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B68" s="1">
-        <v>23.83</v>
-      </c>
-      <c r="C68" s="1">
-        <v>108.1</v>
-      </c>
-      <c r="D68" s="1">
-        <v>2024</v>
-      </c>
-      <c r="E68" s="3">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A70" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B70" s="1">
+        <v>23.83</v>
+      </c>
+      <c r="C70" s="1">
+        <v>108.1</v>
+      </c>
+      <c r="D70" s="1">
+        <v>2024</v>
+      </c>
+      <c r="E70" s="3">
         <v>45458</v>
       </c>
-      <c r="F68" s="1">
+      <c r="F70" s="1">
         <v>75</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A69" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B69" s="1">
-        <v>23.83</v>
-      </c>
-      <c r="C69" s="1">
-        <v>108.1</v>
-      </c>
-      <c r="D69" s="1">
-        <v>2024</v>
-      </c>
-      <c r="E69" s="3">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A71" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B71" s="1">
+        <v>23.83</v>
+      </c>
+      <c r="C71" s="1">
+        <v>108.1</v>
+      </c>
+      <c r="D71" s="1">
+        <v>2024</v>
+      </c>
+      <c r="E71" s="3">
         <v>45482</v>
       </c>
-      <c r="F69" s="1">
+      <c r="F71" s="1">
         <v>79</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A70" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B70" s="5">
-        <v>25.45</v>
-      </c>
-      <c r="C70" s="5">
-        <v>110.8</v>
-      </c>
-      <c r="D70" s="5">
-        <v>2022</v>
-      </c>
-      <c r="E70" s="6">
-        <v>44654</v>
-      </c>
-      <c r="F70" s="7">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A71" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B71" s="5">
-        <v>25.45</v>
-      </c>
-      <c r="C71" s="5">
-        <v>110.8</v>
-      </c>
-      <c r="D71" s="5">
-        <v>2022</v>
-      </c>
-      <c r="E71" s="6">
-        <v>44661</v>
-      </c>
-      <c r="F71" s="7">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
         <v>8</v>
       </c>
@@ -1924,13 +1930,13 @@
         <v>2022</v>
       </c>
       <c r="E72" s="6">
-        <v>44668</v>
+        <v>44646</v>
       </c>
       <c r="F72" s="7">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A73" s="2" t="s">
         <v>8</v>
       </c>
@@ -1944,13 +1950,14 @@
         <v>2022</v>
       </c>
       <c r="E73" s="6">
-        <v>44675</v>
+        <v>44654</v>
       </c>
       <c r="F73" s="7">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+      <c r="J73" s="8"/>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A74" s="2" t="s">
         <v>8</v>
       </c>
@@ -1964,13 +1971,13 @@
         <v>2022</v>
       </c>
       <c r="E74" s="6">
-        <v>44685</v>
+        <v>44661</v>
       </c>
       <c r="F74" s="7">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A75" s="2" t="s">
         <v>8</v>
       </c>
@@ -1984,13 +1991,13 @@
         <v>2022</v>
       </c>
       <c r="E75" s="6">
-        <v>44694</v>
+        <v>44668</v>
       </c>
       <c r="F75" s="7">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A76" s="2" t="s">
         <v>8</v>
       </c>
@@ -2004,13 +2011,13 @@
         <v>2022</v>
       </c>
       <c r="E76" s="6">
-        <v>44702</v>
+        <v>44675</v>
       </c>
       <c r="F76" s="7">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A77" s="2" t="s">
         <v>8</v>
       </c>
@@ -2024,9 +2031,69 @@
         <v>2022</v>
       </c>
       <c r="E77" s="6">
+        <v>44685</v>
+      </c>
+      <c r="F77" s="7">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A78" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B78" s="5">
+        <v>25.45</v>
+      </c>
+      <c r="C78" s="5">
+        <v>110.8</v>
+      </c>
+      <c r="D78" s="5">
+        <v>2022</v>
+      </c>
+      <c r="E78" s="6">
+        <v>44694</v>
+      </c>
+      <c r="F78" s="7">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A79" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B79" s="5">
+        <v>25.45</v>
+      </c>
+      <c r="C79" s="5">
+        <v>110.8</v>
+      </c>
+      <c r="D79" s="5">
+        <v>2022</v>
+      </c>
+      <c r="E79" s="6">
+        <v>44702</v>
+      </c>
+      <c r="F79" s="7">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A80" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B80" s="5">
+        <v>25.45</v>
+      </c>
+      <c r="C80" s="5">
+        <v>110.8</v>
+      </c>
+      <c r="D80" s="5">
+        <v>2022</v>
+      </c>
+      <c r="E80" s="6">
         <v>44711</v>
       </c>
-      <c r="F77" s="7">
+      <c r="F80" s="7">
         <v>75</v>
       </c>
     </row>

</xml_diff>